<commit_message>
Added DECISIONS, and updated LOG and purchase tracker
</commit_message>
<xml_diff>
--- a/admin/EDF_Purchasing_Tracker.xlsx
+++ b/admin/EDF_Purchasing_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Speed\Projects\edf-testbed\admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D362F9-A9D6-485C-AE5D-7A6F4083476D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6978EF25-A202-418F-8A7F-4C055DCD5517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="218">
   <si>
     <t>Chin-Inlet EDF UAV Testbed - Purchasing Tracker</t>
   </si>
@@ -732,7 +732,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -779,12 +779,6 @@
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -918,21 +912,14 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD5F0D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -1495,9 +1482,7 @@
       <c r="I2" s="12">
         <v>46275</v>
       </c>
-      <c r="J2" s="12" t="s">
-        <v>197</v>
-      </c>
+      <c r="J2" s="12"/>
       <c r="K2" s="8" t="s">
         <v>45</v>
       </c>
@@ -1532,7 +1517,9 @@
       <c r="I3" s="12">
         <v>46275</v>
       </c>
-      <c r="J3" s="12"/>
+      <c r="J3" s="12">
+        <v>46278</v>
+      </c>
       <c r="K3" s="8" t="s">
         <v>48</v>
       </c>
@@ -1567,7 +1554,9 @@
       <c r="I4" s="12">
         <v>46275</v>
       </c>
-      <c r="J4" s="12"/>
+      <c r="J4" s="12">
+        <v>46278</v>
+      </c>
       <c r="K4" s="8" t="s">
         <v>51</v>
       </c>
@@ -1629,7 +1618,9 @@
       <c r="I6" s="12">
         <v>46275</v>
       </c>
-      <c r="J6" s="12"/>
+      <c r="J6" s="12">
+        <v>46278</v>
+      </c>
       <c r="K6" s="8" t="s">
         <v>56</v>
       </c>
@@ -1663,7 +1654,9 @@
       <c r="I7" s="12">
         <v>46275</v>
       </c>
-      <c r="J7" s="12"/>
+      <c r="J7" s="12">
+        <v>46278</v>
+      </c>
       <c r="K7" s="8" t="s">
         <v>59</v>
       </c>
@@ -1697,7 +1690,9 @@
       <c r="I8" s="12">
         <v>46275</v>
       </c>
-      <c r="J8" s="12"/>
+      <c r="J8" s="12">
+        <v>46278</v>
+      </c>
       <c r="K8" s="8" t="s">
         <v>61</v>
       </c>
@@ -2236,7 +2231,9 @@
       <c r="I27" s="12">
         <v>46275</v>
       </c>
-      <c r="J27" s="12"/>
+      <c r="J27" s="12">
+        <v>46279</v>
+      </c>
       <c r="K27" s="8" t="s">
         <v>117</v>
       </c>
@@ -2270,7 +2267,9 @@
       <c r="I28" s="12">
         <v>46275</v>
       </c>
-      <c r="J28" s="12"/>
+      <c r="J28" s="12">
+        <v>46278</v>
+      </c>
       <c r="K28" s="8" t="s">
         <v>118</v>
       </c>
@@ -2584,7 +2583,9 @@
       <c r="I39" s="12">
         <v>46275</v>
       </c>
-      <c r="J39" s="12"/>
+      <c r="J39" s="12">
+        <v>46278</v>
+      </c>
       <c r="K39" s="8" t="s">
         <v>149</v>
       </c>
@@ -2903,7 +2904,9 @@
       <c r="I50" s="12">
         <v>46275</v>
       </c>
-      <c r="J50" s="12"/>
+      <c r="J50" s="12">
+        <v>46278</v>
+      </c>
       <c r="K50" s="8"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
@@ -3079,13 +3082,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K54" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <conditionalFormatting sqref="A2:K26 A51:F54 A48:C50 E48:F50 A44:F47 G44:K54 A28:K43 A27:C27 E27:K27 D50">
-    <cfRule type="expression" dxfId="0" priority="2">
+  <conditionalFormatting sqref="A2:K26 A27:C27 E27:K27 A28:K43 A44:F47 G44:K54 A48:C50 E48:F50 D50 A51:F54">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$A2="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D48">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>$A49="Yes"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>